<commit_message>
Local workbooks: mirror live Instructions wording
.xlsx gets the online snapshot section and client email mentions;
.xlsm gets the desktop equivalents. Backlog and handoff updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Project Schedules.xlsx
+++ b/Project Schedules.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\gantt-chart-varennes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68C66CEF-C2A5-4DB9-AF6C-82293D00931B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ECDF4E4-929C-4D9D-A46B-A8E7862198B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6240" yWindow="6240" windowWidth="32400" windowHeight="19395" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projects" sheetId="14" r:id="rId1"/>
@@ -123,7 +123,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="102">
   <si>
     <t>Atlantic Packaging Network Install</t>
   </si>
@@ -348,9 +348,6 @@
     <t>•</t>
   </si>
   <si>
-    <t>Projects tab: one line per project with client, project manager, start, finish, progress and status. Click a project name to open its tab.</t>
-  </si>
-  <si>
     <t>One tab per project: the Gantt chart. The '◄ All projects' link at the top of the chart takes you back to the Projects tab.</t>
   </si>
   <si>
@@ -387,9 +384,6 @@
     <t>1.  Go to the Projects tab and click Run New Project.</t>
   </si>
   <si>
-    <t>2.  Enter the project name and start date (for example 2026-11-02); client and project manager are optional. Click Run.</t>
-  </si>
-  <si>
     <t>Run Add Task: select a task first; the new task goes right below it. Select a section header instead and it goes at the end of that section.</t>
   </si>
   <si>
@@ -418,6 +412,24 @@
   </si>
   <si>
     <t>Client Email</t>
+  </si>
+  <si>
+    <t>Projects tab: one line per project with client, project manager, start, finish, progress, status and client email. Click a project name to open its tab.</t>
+  </si>
+  <si>
+    <t>2.  Enter the project name and start date (for example 2026-11-02); client, project manager and client email are optional. Click Run.</t>
+  </si>
+  <si>
+    <t>Send the client a snapshot</t>
+  </si>
+  <si>
+    <t>On the project's tab, click Run Email Snapshot to Client. Within about two minutes the person who clicked gets an email with a PDF and an Excel copy of just that project, ready to forward to the client.</t>
+  </si>
+  <si>
+    <t>The snapshot is a frozen copy as of today: no other projects, no formulas, no invoice markers or internal controls.</t>
+  </si>
+  <si>
+    <t>The client's address comes from the Client Email column on the Projects tab; fill it in so the email tells you where to send it.</t>
   </si>
 </sst>
 </file>
@@ -1288,6 +1300,21 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="166" fontId="11" fillId="17" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="17" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -1297,23 +1324,8 @@
     <xf numFmtId="165" fontId="0" fillId="7" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="17" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="17" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -2008,7 +2020,7 @@
         <v>68</v>
       </c>
       <c r="K5" s="98" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.25">
@@ -10054,7 +10066,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{037E1AD6-8148-4020-9FCE-F76B4C0D8F5B}">
-  <dimension ref="A1:D200"/>
+  <dimension ref="A1:D205"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="109" customWidth="1"/>
@@ -10102,7 +10114,7 @@
         <v>73</v>
       </c>
       <c r="C5" s="115" t="s">
-        <v>74</v>
+        <v>96</v>
       </c>
       <c r="D5"/>
     </row>
@@ -10112,7 +10124,7 @@
         <v>73</v>
       </c>
       <c r="C6" s="115" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D6"/>
     </row>
@@ -10122,7 +10134,7 @@
         <v>73</v>
       </c>
       <c r="C7" s="115" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D7"/>
     </row>
@@ -10135,7 +10147,7 @@
     <row r="9" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9"/>
       <c r="B9" s="113" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C9" s="111"/>
       <c r="D9"/>
@@ -10144,7 +10156,7 @@
       <c r="A10"/>
       <c r="B10" s="111"/>
       <c r="C10" s="115" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D10"/>
     </row>
@@ -10152,7 +10164,7 @@
       <c r="A11"/>
       <c r="B11" s="111"/>
       <c r="C11" s="115" t="s">
-        <v>87</v>
+        <v>97</v>
       </c>
       <c r="D11"/>
     </row>
@@ -10160,7 +10172,7 @@
       <c r="A12"/>
       <c r="B12" s="111"/>
       <c r="C12" s="115" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D12"/>
     </row>
@@ -10173,7 +10185,7 @@
     <row r="14" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14"/>
       <c r="B14" s="113" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C14" s="111"/>
       <c r="D14"/>
@@ -10184,7 +10196,7 @@
         <v>73</v>
       </c>
       <c r="C15" s="115" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="D15"/>
     </row>
@@ -10194,7 +10206,7 @@
         <v>73</v>
       </c>
       <c r="C16" s="115" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D16"/>
     </row>
@@ -10204,7 +10216,7 @@
         <v>73</v>
       </c>
       <c r="C17" s="115" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D17"/>
     </row>
@@ -10214,7 +10226,7 @@
         <v>73</v>
       </c>
       <c r="C18" s="115" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D18"/>
     </row>
@@ -10224,7 +10236,7 @@
         <v>73</v>
       </c>
       <c r="C19" s="115" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D19"/>
     </row>
@@ -10237,7 +10249,7 @@
     <row r="21" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21"/>
       <c r="B21" s="113" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C21" s="111"/>
       <c r="D21"/>
@@ -10248,7 +10260,7 @@
         <v>73</v>
       </c>
       <c r="C22" s="115" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="D22"/>
     </row>
@@ -10258,7 +10270,7 @@
         <v>73</v>
       </c>
       <c r="C23" s="115" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D23"/>
     </row>
@@ -10271,7 +10283,7 @@
     <row r="25" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25"/>
       <c r="B25" s="113" t="s">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="C25" s="111"/>
       <c r="D25"/>
@@ -10282,7 +10294,7 @@
         <v>73</v>
       </c>
       <c r="C26" s="115" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="D26"/>
     </row>
@@ -10292,82 +10304,96 @@
         <v>73</v>
       </c>
       <c r="C27" s="115" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="D27"/>
     </row>
-    <row r="28" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A28"/>
       <c r="B28" s="114" t="s">
         <v>73</v>
       </c>
       <c r="C28" s="115" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="D28"/>
     </row>
-    <row r="29" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" ht="8.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29"/>
-      <c r="B29" s="114" t="s">
-        <v>73</v>
-      </c>
-      <c r="C29" s="115" t="s">
-        <v>95</v>
-      </c>
+      <c r="B29" s="111"/>
+      <c r="C29" s="111"/>
       <c r="D29"/>
     </row>
-    <row r="30" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30"/>
-      <c r="B30" s="114" t="s">
-        <v>73</v>
-      </c>
-      <c r="C30" s="115" t="s">
-        <v>85</v>
-      </c>
+      <c r="B30" s="113" t="s">
+        <v>82</v>
+      </c>
+      <c r="C30" s="111"/>
       <c r="D30"/>
     </row>
-    <row r="31" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A31"/>
       <c r="B31" s="114" t="s">
         <v>73</v>
       </c>
       <c r="C31" s="115" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="D31"/>
     </row>
     <row r="32" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A32"/>
+      <c r="B32" s="114" t="s">
+        <v>73</v>
+      </c>
+      <c r="C32" s="115" t="s">
+        <v>92</v>
+      </c>
       <c r="D32"/>
     </row>
     <row r="33" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A33"/>
-      <c r="B33"/>
-      <c r="C33"/>
+      <c r="B33" s="114" t="s">
+        <v>73</v>
+      </c>
+      <c r="C33" s="115" t="s">
+        <v>83</v>
+      </c>
       <c r="D33"/>
     </row>
-    <row r="34" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A34"/>
-      <c r="B34"/>
-      <c r="C34"/>
+      <c r="B34" s="114" t="s">
+        <v>73</v>
+      </c>
+      <c r="C34" s="115" t="s">
+        <v>93</v>
+      </c>
       <c r="D34"/>
     </row>
-    <row r="35" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A35"/>
-      <c r="B35"/>
-      <c r="C35"/>
+      <c r="B35" s="114" t="s">
+        <v>73</v>
+      </c>
+      <c r="C35" s="115" t="s">
+        <v>84</v>
+      </c>
       <c r="D35"/>
     </row>
     <row r="36" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A36"/>
-      <c r="B36"/>
-      <c r="C36"/>
+      <c r="B36" s="114" t="s">
+        <v>73</v>
+      </c>
+      <c r="C36" s="115" t="s">
+        <v>94</v>
+      </c>
       <c r="D36"/>
     </row>
     <row r="37" spans="1:4" ht="15" x14ac:dyDescent="0.25">
       <c r="A37"/>
-      <c r="B37"/>
-      <c r="C37"/>
       <c r="D37"/>
     </row>
     <row r="38" spans="1:4" ht="15" x14ac:dyDescent="0.25">
@@ -11347,6 +11373,36 @@
       <c r="B200"/>
       <c r="C200"/>
       <c r="D200"/>
+    </row>
+    <row r="201" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A201"/>
+      <c r="B201"/>
+      <c r="C201"/>
+      <c r="D201"/>
+    </row>
+    <row r="202" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A202"/>
+      <c r="B202"/>
+      <c r="C202"/>
+      <c r="D202"/>
+    </row>
+    <row r="203" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A203"/>
+      <c r="B203"/>
+      <c r="C203"/>
+      <c r="D203"/>
+    </row>
+    <row r="204" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A204"/>
+      <c r="B204"/>
+      <c r="C204"/>
+      <c r="D204"/>
+    </row>
+    <row r="205" spans="1:4" ht="15" x14ac:dyDescent="0.25">
+      <c r="A205"/>
+      <c r="B205"/>
+      <c r="C205"/>
+      <c r="D205"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -11382,15 +11438,15 @@
       <c r="E1" s="4"/>
       <c r="F1" s="77"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="124" t="str">
+      <c r="I1" s="127" t="str">
         <f>HYPERLINK("#'Projects'!A1","◄ All projects")</f>
         <v>◄ All projects</v>
       </c>
-      <c r="J1" s="124"/>
-      <c r="K1" s="124"/>
-      <c r="L1" s="124"/>
-      <c r="M1" s="124"/>
-      <c r="N1" s="124"/>
+      <c r="J1" s="127"/>
+      <c r="K1" s="127"/>
+      <c r="L1" s="127"/>
+      <c r="M1" s="127"/>
+      <c r="N1" s="127"/>
       <c r="O1" s="116"/>
       <c r="P1" s="116"/>
       <c r="Q1" s="116"/>
@@ -11446,186 +11502,186 @@
       <c r="E4" s="7">
         <v>1</v>
       </c>
-      <c r="I4" s="119">
+      <c r="I4" s="124">
         <f>I5</f>
         <v>45313</v>
       </c>
-      <c r="J4" s="120"/>
-      <c r="K4" s="120"/>
-      <c r="L4" s="120"/>
-      <c r="M4" s="120"/>
-      <c r="N4" s="120"/>
-      <c r="O4" s="121"/>
-      <c r="P4" s="119">
+      <c r="J4" s="125"/>
+      <c r="K4" s="125"/>
+      <c r="L4" s="125"/>
+      <c r="M4" s="125"/>
+      <c r="N4" s="125"/>
+      <c r="O4" s="126"/>
+      <c r="P4" s="124">
         <f>P5</f>
         <v>45320</v>
       </c>
-      <c r="Q4" s="120"/>
-      <c r="R4" s="120"/>
-      <c r="S4" s="120"/>
-      <c r="T4" s="120"/>
-      <c r="U4" s="120"/>
-      <c r="V4" s="121"/>
-      <c r="W4" s="119">
+      <c r="Q4" s="125"/>
+      <c r="R4" s="125"/>
+      <c r="S4" s="125"/>
+      <c r="T4" s="125"/>
+      <c r="U4" s="125"/>
+      <c r="V4" s="126"/>
+      <c r="W4" s="124">
         <f>W5</f>
         <v>45327</v>
       </c>
-      <c r="X4" s="120"/>
-      <c r="Y4" s="120"/>
-      <c r="Z4" s="120"/>
-      <c r="AA4" s="120"/>
-      <c r="AB4" s="120"/>
-      <c r="AC4" s="121"/>
-      <c r="AD4" s="119">
+      <c r="X4" s="125"/>
+      <c r="Y4" s="125"/>
+      <c r="Z4" s="125"/>
+      <c r="AA4" s="125"/>
+      <c r="AB4" s="125"/>
+      <c r="AC4" s="126"/>
+      <c r="AD4" s="124">
         <f>AD5</f>
         <v>45334</v>
       </c>
-      <c r="AE4" s="120"/>
-      <c r="AF4" s="120"/>
-      <c r="AG4" s="120"/>
-      <c r="AH4" s="120"/>
-      <c r="AI4" s="120"/>
-      <c r="AJ4" s="121"/>
-      <c r="AK4" s="119">
+      <c r="AE4" s="125"/>
+      <c r="AF4" s="125"/>
+      <c r="AG4" s="125"/>
+      <c r="AH4" s="125"/>
+      <c r="AI4" s="125"/>
+      <c r="AJ4" s="126"/>
+      <c r="AK4" s="124">
         <f>AK5</f>
         <v>45341</v>
       </c>
-      <c r="AL4" s="120"/>
-      <c r="AM4" s="120"/>
-      <c r="AN4" s="120"/>
-      <c r="AO4" s="120"/>
-      <c r="AP4" s="120"/>
-      <c r="AQ4" s="121"/>
-      <c r="AR4" s="119">
+      <c r="AL4" s="125"/>
+      <c r="AM4" s="125"/>
+      <c r="AN4" s="125"/>
+      <c r="AO4" s="125"/>
+      <c r="AP4" s="125"/>
+      <c r="AQ4" s="126"/>
+      <c r="AR4" s="124">
         <f>AR5</f>
         <v>45348</v>
       </c>
-      <c r="AS4" s="120"/>
-      <c r="AT4" s="120"/>
-      <c r="AU4" s="120"/>
-      <c r="AV4" s="120"/>
-      <c r="AW4" s="120"/>
-      <c r="AX4" s="121"/>
-      <c r="AY4" s="119">
+      <c r="AS4" s="125"/>
+      <c r="AT4" s="125"/>
+      <c r="AU4" s="125"/>
+      <c r="AV4" s="125"/>
+      <c r="AW4" s="125"/>
+      <c r="AX4" s="126"/>
+      <c r="AY4" s="124">
         <f>AY5</f>
         <v>45355</v>
       </c>
-      <c r="AZ4" s="120"/>
-      <c r="BA4" s="120"/>
-      <c r="BB4" s="120"/>
-      <c r="BC4" s="120"/>
-      <c r="BD4" s="120"/>
-      <c r="BE4" s="121"/>
-      <c r="BF4" s="119">
+      <c r="AZ4" s="125"/>
+      <c r="BA4" s="125"/>
+      <c r="BB4" s="125"/>
+      <c r="BC4" s="125"/>
+      <c r="BD4" s="125"/>
+      <c r="BE4" s="126"/>
+      <c r="BF4" s="124">
         <f>BF5</f>
         <v>45362</v>
       </c>
-      <c r="BG4" s="120"/>
-      <c r="BH4" s="120"/>
-      <c r="BI4" s="120"/>
-      <c r="BJ4" s="120"/>
-      <c r="BK4" s="120"/>
-      <c r="BL4" s="121"/>
-      <c r="BM4" s="119">
+      <c r="BG4" s="125"/>
+      <c r="BH4" s="125"/>
+      <c r="BI4" s="125"/>
+      <c r="BJ4" s="125"/>
+      <c r="BK4" s="125"/>
+      <c r="BL4" s="126"/>
+      <c r="BM4" s="124">
         <f>BM5</f>
         <v>45369</v>
       </c>
-      <c r="BN4" s="120"/>
-      <c r="BO4" s="120"/>
-      <c r="BP4" s="120"/>
-      <c r="BQ4" s="120"/>
-      <c r="BR4" s="120"/>
-      <c r="BS4" s="121"/>
-      <c r="BT4" s="119">
+      <c r="BN4" s="125"/>
+      <c r="BO4" s="125"/>
+      <c r="BP4" s="125"/>
+      <c r="BQ4" s="125"/>
+      <c r="BR4" s="125"/>
+      <c r="BS4" s="126"/>
+      <c r="BT4" s="124">
         <f>BT5</f>
         <v>45376</v>
       </c>
-      <c r="BU4" s="120"/>
-      <c r="BV4" s="120"/>
-      <c r="BW4" s="120"/>
-      <c r="BX4" s="120"/>
-      <c r="BY4" s="120"/>
-      <c r="BZ4" s="121"/>
-      <c r="CA4" s="119">
+      <c r="BU4" s="125"/>
+      <c r="BV4" s="125"/>
+      <c r="BW4" s="125"/>
+      <c r="BX4" s="125"/>
+      <c r="BY4" s="125"/>
+      <c r="BZ4" s="126"/>
+      <c r="CA4" s="124">
         <f>CA5</f>
         <v>45383</v>
       </c>
-      <c r="CB4" s="120"/>
-      <c r="CC4" s="120"/>
-      <c r="CD4" s="120"/>
-      <c r="CE4" s="120"/>
-      <c r="CF4" s="120"/>
-      <c r="CG4" s="121"/>
-      <c r="CH4" s="119">
+      <c r="CB4" s="125"/>
+      <c r="CC4" s="125"/>
+      <c r="CD4" s="125"/>
+      <c r="CE4" s="125"/>
+      <c r="CF4" s="125"/>
+      <c r="CG4" s="126"/>
+      <c r="CH4" s="124">
         <f>CH5</f>
         <v>45390</v>
       </c>
-      <c r="CI4" s="120"/>
-      <c r="CJ4" s="120"/>
-      <c r="CK4" s="120"/>
-      <c r="CL4" s="120"/>
-      <c r="CM4" s="120"/>
-      <c r="CN4" s="121"/>
-      <c r="CO4" s="119">
+      <c r="CI4" s="125"/>
+      <c r="CJ4" s="125"/>
+      <c r="CK4" s="125"/>
+      <c r="CL4" s="125"/>
+      <c r="CM4" s="125"/>
+      <c r="CN4" s="126"/>
+      <c r="CO4" s="124">
         <f>CO5</f>
         <v>45397</v>
       </c>
-      <c r="CP4" s="120"/>
-      <c r="CQ4" s="120"/>
-      <c r="CR4" s="120"/>
-      <c r="CS4" s="120"/>
-      <c r="CT4" s="120"/>
-      <c r="CU4" s="121"/>
-      <c r="CV4" s="119">
+      <c r="CP4" s="125"/>
+      <c r="CQ4" s="125"/>
+      <c r="CR4" s="125"/>
+      <c r="CS4" s="125"/>
+      <c r="CT4" s="125"/>
+      <c r="CU4" s="126"/>
+      <c r="CV4" s="124">
         <f>CV5</f>
         <v>45404</v>
       </c>
-      <c r="CW4" s="120"/>
-      <c r="CX4" s="120"/>
-      <c r="CY4" s="120"/>
-      <c r="CZ4" s="120"/>
-      <c r="DA4" s="120"/>
-      <c r="DB4" s="121"/>
-      <c r="DC4" s="119">
+      <c r="CW4" s="125"/>
+      <c r="CX4" s="125"/>
+      <c r="CY4" s="125"/>
+      <c r="CZ4" s="125"/>
+      <c r="DA4" s="125"/>
+      <c r="DB4" s="126"/>
+      <c r="DC4" s="124">
         <f>DC5</f>
         <v>45411</v>
       </c>
-      <c r="DD4" s="120"/>
-      <c r="DE4" s="120"/>
-      <c r="DF4" s="120"/>
-      <c r="DG4" s="120"/>
-      <c r="DH4" s="120"/>
-      <c r="DI4" s="121"/>
-      <c r="DJ4" s="119">
+      <c r="DD4" s="125"/>
+      <c r="DE4" s="125"/>
+      <c r="DF4" s="125"/>
+      <c r="DG4" s="125"/>
+      <c r="DH4" s="125"/>
+      <c r="DI4" s="126"/>
+      <c r="DJ4" s="124">
         <f>DJ5</f>
         <v>45418</v>
       </c>
-      <c r="DK4" s="120"/>
-      <c r="DL4" s="120"/>
-      <c r="DM4" s="120"/>
-      <c r="DN4" s="120"/>
-      <c r="DO4" s="120"/>
-      <c r="DP4" s="121"/>
-      <c r="DQ4" s="119">
+      <c r="DK4" s="125"/>
+      <c r="DL4" s="125"/>
+      <c r="DM4" s="125"/>
+      <c r="DN4" s="125"/>
+      <c r="DO4" s="125"/>
+      <c r="DP4" s="126"/>
+      <c r="DQ4" s="124">
         <f>DQ5</f>
         <v>45425</v>
       </c>
-      <c r="DR4" s="120"/>
-      <c r="DS4" s="120"/>
-      <c r="DT4" s="120"/>
-      <c r="DU4" s="120"/>
-      <c r="DV4" s="120"/>
-      <c r="DW4" s="121"/>
-      <c r="DX4" s="119">
+      <c r="DR4" s="125"/>
+      <c r="DS4" s="125"/>
+      <c r="DT4" s="125"/>
+      <c r="DU4" s="125"/>
+      <c r="DV4" s="125"/>
+      <c r="DW4" s="126"/>
+      <c r="DX4" s="124">
         <f>DX5</f>
         <v>45432</v>
       </c>
-      <c r="DY4" s="120"/>
-      <c r="DZ4" s="120"/>
-      <c r="EA4" s="120"/>
-      <c r="EB4" s="120"/>
-      <c r="EC4" s="120"/>
-      <c r="ED4" s="121"/>
+      <c r="DY4" s="125"/>
+      <c r="DZ4" s="125"/>
+      <c r="EA4" s="125"/>
+      <c r="EB4" s="125"/>
+      <c r="EC4" s="125"/>
+      <c r="ED4" s="126"/>
     </row>
     <row r="5" spans="1:134" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
@@ -17914,16 +17970,16 @@
     <mergeCell ref="CO4:CU4"/>
     <mergeCell ref="CV4:DB4"/>
     <mergeCell ref="BM4:BS4"/>
+    <mergeCell ref="AK4:AQ4"/>
+    <mergeCell ref="AR4:AX4"/>
+    <mergeCell ref="AY4:BE4"/>
+    <mergeCell ref="BF4:BL4"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="I4:O4"/>
     <mergeCell ref="P4:V4"/>
     <mergeCell ref="W4:AC4"/>
     <mergeCell ref="AD4:AJ4"/>
     <mergeCell ref="E3:F3"/>
-    <mergeCell ref="AK4:AQ4"/>
-    <mergeCell ref="AR4:AX4"/>
-    <mergeCell ref="AY4:BE4"/>
-    <mergeCell ref="BF4:BL4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D42">
     <cfRule type="dataBar" priority="42">
@@ -18014,15 +18070,15 @@
       <c r="E1" s="4"/>
       <c r="F1" s="77"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="124" t="str">
+      <c r="I1" s="127" t="str">
         <f>HYPERLINK("#'Projects'!A1","◄ All projects")</f>
         <v>◄ All projects</v>
       </c>
-      <c r="J1" s="124"/>
-      <c r="K1" s="124"/>
-      <c r="L1" s="124"/>
-      <c r="M1" s="124"/>
-      <c r="N1" s="124"/>
+      <c r="J1" s="127"/>
+      <c r="K1" s="127"/>
+      <c r="L1" s="127"/>
+      <c r="M1" s="127"/>
+      <c r="N1" s="127"/>
       <c r="O1" s="116"/>
       <c r="P1" s="116"/>
       <c r="Q1" s="116"/>
@@ -18070,691 +18126,691 @@
       <c r="E4" s="7">
         <v>1</v>
       </c>
-      <c r="I4" s="119">
+      <c r="I4" s="124">
         <f>I5</f>
         <v>45313</v>
       </c>
-      <c r="J4" s="120"/>
-      <c r="K4" s="120"/>
-      <c r="L4" s="120"/>
-      <c r="M4" s="120"/>
-      <c r="N4" s="120"/>
-      <c r="O4" s="121"/>
-      <c r="P4" s="119">
+      <c r="J4" s="125"/>
+      <c r="K4" s="125"/>
+      <c r="L4" s="125"/>
+      <c r="M4" s="125"/>
+      <c r="N4" s="125"/>
+      <c r="O4" s="126"/>
+      <c r="P4" s="124">
         <f>P5</f>
         <v>45320</v>
       </c>
-      <c r="Q4" s="120"/>
-      <c r="R4" s="120"/>
-      <c r="S4" s="120"/>
-      <c r="T4" s="120"/>
-      <c r="U4" s="120"/>
-      <c r="V4" s="121"/>
-      <c r="W4" s="119">
+      <c r="Q4" s="125"/>
+      <c r="R4" s="125"/>
+      <c r="S4" s="125"/>
+      <c r="T4" s="125"/>
+      <c r="U4" s="125"/>
+      <c r="V4" s="126"/>
+      <c r="W4" s="124">
         <f>W5</f>
         <v>45327</v>
       </c>
-      <c r="X4" s="120"/>
-      <c r="Y4" s="120"/>
-      <c r="Z4" s="120"/>
-      <c r="AA4" s="120"/>
-      <c r="AB4" s="120"/>
-      <c r="AC4" s="121"/>
-      <c r="AD4" s="119">
+      <c r="X4" s="125"/>
+      <c r="Y4" s="125"/>
+      <c r="Z4" s="125"/>
+      <c r="AA4" s="125"/>
+      <c r="AB4" s="125"/>
+      <c r="AC4" s="126"/>
+      <c r="AD4" s="124">
         <f>AD5</f>
         <v>45334</v>
       </c>
-      <c r="AE4" s="120"/>
-      <c r="AF4" s="120"/>
-      <c r="AG4" s="120"/>
-      <c r="AH4" s="120"/>
-      <c r="AI4" s="120"/>
-      <c r="AJ4" s="121"/>
-      <c r="AK4" s="119">
+      <c r="AE4" s="125"/>
+      <c r="AF4" s="125"/>
+      <c r="AG4" s="125"/>
+      <c r="AH4" s="125"/>
+      <c r="AI4" s="125"/>
+      <c r="AJ4" s="126"/>
+      <c r="AK4" s="124">
         <f>AK5</f>
         <v>45341</v>
       </c>
-      <c r="AL4" s="120"/>
-      <c r="AM4" s="120"/>
-      <c r="AN4" s="120"/>
-      <c r="AO4" s="120"/>
-      <c r="AP4" s="120"/>
-      <c r="AQ4" s="121"/>
-      <c r="AR4" s="119">
+      <c r="AL4" s="125"/>
+      <c r="AM4" s="125"/>
+      <c r="AN4" s="125"/>
+      <c r="AO4" s="125"/>
+      <c r="AP4" s="125"/>
+      <c r="AQ4" s="126"/>
+      <c r="AR4" s="124">
         <f>AR5</f>
         <v>45348</v>
       </c>
-      <c r="AS4" s="120"/>
-      <c r="AT4" s="120"/>
-      <c r="AU4" s="120"/>
-      <c r="AV4" s="120"/>
-      <c r="AW4" s="120"/>
-      <c r="AX4" s="121"/>
-      <c r="AY4" s="119">
+      <c r="AS4" s="125"/>
+      <c r="AT4" s="125"/>
+      <c r="AU4" s="125"/>
+      <c r="AV4" s="125"/>
+      <c r="AW4" s="125"/>
+      <c r="AX4" s="126"/>
+      <c r="AY4" s="124">
         <f>AY5</f>
         <v>45355</v>
       </c>
-      <c r="AZ4" s="120"/>
-      <c r="BA4" s="120"/>
-      <c r="BB4" s="120"/>
-      <c r="BC4" s="120"/>
-      <c r="BD4" s="120"/>
-      <c r="BE4" s="121"/>
-      <c r="BF4" s="119">
+      <c r="AZ4" s="125"/>
+      <c r="BA4" s="125"/>
+      <c r="BB4" s="125"/>
+      <c r="BC4" s="125"/>
+      <c r="BD4" s="125"/>
+      <c r="BE4" s="126"/>
+      <c r="BF4" s="124">
         <f>BF5</f>
         <v>45362</v>
       </c>
-      <c r="BG4" s="120"/>
-      <c r="BH4" s="120"/>
-      <c r="BI4" s="120"/>
-      <c r="BJ4" s="120"/>
-      <c r="BK4" s="120"/>
-      <c r="BL4" s="121"/>
-      <c r="BM4" s="119">
+      <c r="BG4" s="125"/>
+      <c r="BH4" s="125"/>
+      <c r="BI4" s="125"/>
+      <c r="BJ4" s="125"/>
+      <c r="BK4" s="125"/>
+      <c r="BL4" s="126"/>
+      <c r="BM4" s="124">
         <f>BM5</f>
         <v>45369</v>
       </c>
-      <c r="BN4" s="120"/>
-      <c r="BO4" s="120"/>
-      <c r="BP4" s="120"/>
-      <c r="BQ4" s="120"/>
-      <c r="BR4" s="120"/>
-      <c r="BS4" s="121"/>
-      <c r="BT4" s="119">
+      <c r="BN4" s="125"/>
+      <c r="BO4" s="125"/>
+      <c r="BP4" s="125"/>
+      <c r="BQ4" s="125"/>
+      <c r="BR4" s="125"/>
+      <c r="BS4" s="126"/>
+      <c r="BT4" s="124">
         <f>BT5</f>
         <v>45376</v>
       </c>
-      <c r="BU4" s="120"/>
-      <c r="BV4" s="120"/>
-      <c r="BW4" s="120"/>
-      <c r="BX4" s="120"/>
-      <c r="BY4" s="120"/>
-      <c r="BZ4" s="121"/>
-      <c r="CA4" s="119">
+      <c r="BU4" s="125"/>
+      <c r="BV4" s="125"/>
+      <c r="BW4" s="125"/>
+      <c r="BX4" s="125"/>
+      <c r="BY4" s="125"/>
+      <c r="BZ4" s="126"/>
+      <c r="CA4" s="124">
         <f>CA5</f>
         <v>45383</v>
       </c>
-      <c r="CB4" s="120"/>
-      <c r="CC4" s="120"/>
-      <c r="CD4" s="120"/>
-      <c r="CE4" s="120"/>
-      <c r="CF4" s="120"/>
-      <c r="CG4" s="121"/>
-      <c r="CH4" s="119">
+      <c r="CB4" s="125"/>
+      <c r="CC4" s="125"/>
+      <c r="CD4" s="125"/>
+      <c r="CE4" s="125"/>
+      <c r="CF4" s="125"/>
+      <c r="CG4" s="126"/>
+      <c r="CH4" s="124">
         <f>CH5</f>
         <v>45390</v>
       </c>
-      <c r="CI4" s="120"/>
-      <c r="CJ4" s="120"/>
-      <c r="CK4" s="120"/>
-      <c r="CL4" s="120"/>
-      <c r="CM4" s="120"/>
-      <c r="CN4" s="121"/>
-      <c r="CO4" s="119">
+      <c r="CI4" s="125"/>
+      <c r="CJ4" s="125"/>
+      <c r="CK4" s="125"/>
+      <c r="CL4" s="125"/>
+      <c r="CM4" s="125"/>
+      <c r="CN4" s="126"/>
+      <c r="CO4" s="124">
         <f>CO5</f>
         <v>45397</v>
       </c>
-      <c r="CP4" s="120"/>
-      <c r="CQ4" s="120"/>
-      <c r="CR4" s="120"/>
-      <c r="CS4" s="120"/>
-      <c r="CT4" s="120"/>
-      <c r="CU4" s="121"/>
-      <c r="CV4" s="119">
+      <c r="CP4" s="125"/>
+      <c r="CQ4" s="125"/>
+      <c r="CR4" s="125"/>
+      <c r="CS4" s="125"/>
+      <c r="CT4" s="125"/>
+      <c r="CU4" s="126"/>
+      <c r="CV4" s="124">
         <f>CV5</f>
         <v>45404</v>
       </c>
-      <c r="CW4" s="120"/>
-      <c r="CX4" s="120"/>
-      <c r="CY4" s="120"/>
-      <c r="CZ4" s="120"/>
-      <c r="DA4" s="120"/>
-      <c r="DB4" s="121"/>
-      <c r="DC4" s="119">
+      <c r="CW4" s="125"/>
+      <c r="CX4" s="125"/>
+      <c r="CY4" s="125"/>
+      <c r="CZ4" s="125"/>
+      <c r="DA4" s="125"/>
+      <c r="DB4" s="126"/>
+      <c r="DC4" s="124">
         <f>DC5</f>
         <v>45411</v>
       </c>
-      <c r="DD4" s="120"/>
-      <c r="DE4" s="120"/>
-      <c r="DF4" s="120"/>
-      <c r="DG4" s="120"/>
-      <c r="DH4" s="120"/>
-      <c r="DI4" s="121"/>
-      <c r="DJ4" s="119">
+      <c r="DD4" s="125"/>
+      <c r="DE4" s="125"/>
+      <c r="DF4" s="125"/>
+      <c r="DG4" s="125"/>
+      <c r="DH4" s="125"/>
+      <c r="DI4" s="126"/>
+      <c r="DJ4" s="124">
         <f>DJ5</f>
         <v>45418</v>
       </c>
-      <c r="DK4" s="120"/>
-      <c r="DL4" s="120"/>
-      <c r="DM4" s="120"/>
-      <c r="DN4" s="120"/>
-      <c r="DO4" s="120"/>
-      <c r="DP4" s="121"/>
-      <c r="DQ4" s="119">
+      <c r="DK4" s="125"/>
+      <c r="DL4" s="125"/>
+      <c r="DM4" s="125"/>
+      <c r="DN4" s="125"/>
+      <c r="DO4" s="125"/>
+      <c r="DP4" s="126"/>
+      <c r="DQ4" s="124">
         <f>DQ5</f>
         <v>45425</v>
       </c>
-      <c r="DR4" s="120"/>
-      <c r="DS4" s="120"/>
-      <c r="DT4" s="120"/>
-      <c r="DU4" s="120"/>
-      <c r="DV4" s="120"/>
-      <c r="DW4" s="121"/>
-      <c r="DX4" s="119">
+      <c r="DR4" s="125"/>
+      <c r="DS4" s="125"/>
+      <c r="DT4" s="125"/>
+      <c r="DU4" s="125"/>
+      <c r="DV4" s="125"/>
+      <c r="DW4" s="126"/>
+      <c r="DX4" s="124">
         <f>DX5</f>
         <v>45432</v>
       </c>
-      <c r="DY4" s="120"/>
-      <c r="DZ4" s="120"/>
-      <c r="EA4" s="120"/>
-      <c r="EB4" s="120"/>
-      <c r="EC4" s="120"/>
-      <c r="ED4" s="121"/>
+      <c r="DY4" s="125"/>
+      <c r="DZ4" s="125"/>
+      <c r="EA4" s="125"/>
+      <c r="EB4" s="125"/>
+      <c r="EC4" s="125"/>
+      <c r="ED4" s="126"/>
     </row>
     <row r="5" spans="1:134" x14ac:dyDescent="0.25">
       <c r="A5" s="6"/>
       <c r="G5" s="6"/>
-      <c r="I5" s="125">
+      <c r="I5" s="119">
         <f>E2-WEEKDAY(E2,1)+2+7*(E4-1)</f>
         <v>45313</v>
       </c>
-      <c r="J5" s="126">
+      <c r="J5" s="120">
         <f>I5+1</f>
         <v>45314</v>
       </c>
-      <c r="K5" s="126">
+      <c r="K5" s="120">
         <f t="shared" ref="K5:AX5" si="0">J5+1</f>
         <v>45315</v>
       </c>
-      <c r="L5" s="126">
+      <c r="L5" s="120">
         <f t="shared" si="0"/>
         <v>45316</v>
       </c>
-      <c r="M5" s="126">
+      <c r="M5" s="120">
         <f t="shared" si="0"/>
         <v>45317</v>
       </c>
-      <c r="N5" s="126">
+      <c r="N5" s="120">
         <f t="shared" si="0"/>
         <v>45318</v>
       </c>
-      <c r="O5" s="127">
+      <c r="O5" s="121">
         <f t="shared" si="0"/>
         <v>45319</v>
       </c>
-      <c r="P5" s="125">
+      <c r="P5" s="119">
         <f>O5+1</f>
         <v>45320</v>
       </c>
-      <c r="Q5" s="126">
+      <c r="Q5" s="120">
         <f>P5+1</f>
         <v>45321</v>
       </c>
-      <c r="R5" s="126">
+      <c r="R5" s="120">
         <f t="shared" si="0"/>
         <v>45322</v>
       </c>
-      <c r="S5" s="126">
+      <c r="S5" s="120">
         <f t="shared" si="0"/>
         <v>45323</v>
       </c>
-      <c r="T5" s="126">
+      <c r="T5" s="120">
         <f t="shared" si="0"/>
         <v>45324</v>
       </c>
-      <c r="U5" s="126">
+      <c r="U5" s="120">
         <f t="shared" si="0"/>
         <v>45325</v>
       </c>
-      <c r="V5" s="127">
+      <c r="V5" s="121">
         <f t="shared" si="0"/>
         <v>45326</v>
       </c>
-      <c r="W5" s="125">
+      <c r="W5" s="119">
         <f>V5+1</f>
         <v>45327</v>
       </c>
-      <c r="X5" s="126">
+      <c r="X5" s="120">
         <f>W5+1</f>
         <v>45328</v>
       </c>
-      <c r="Y5" s="126">
+      <c r="Y5" s="120">
         <f t="shared" si="0"/>
         <v>45329</v>
       </c>
-      <c r="Z5" s="126">
+      <c r="Z5" s="120">
         <f t="shared" si="0"/>
         <v>45330</v>
       </c>
-      <c r="AA5" s="126">
+      <c r="AA5" s="120">
         <f t="shared" si="0"/>
         <v>45331</v>
       </c>
-      <c r="AB5" s="126">
+      <c r="AB5" s="120">
         <f t="shared" si="0"/>
         <v>45332</v>
       </c>
-      <c r="AC5" s="127">
+      <c r="AC5" s="121">
         <f t="shared" si="0"/>
         <v>45333</v>
       </c>
-      <c r="AD5" s="125">
+      <c r="AD5" s="119">
         <f>AC5+1</f>
         <v>45334</v>
       </c>
-      <c r="AE5" s="126">
+      <c r="AE5" s="120">
         <f>AD5+1</f>
         <v>45335</v>
       </c>
-      <c r="AF5" s="126">
+      <c r="AF5" s="120">
         <f t="shared" si="0"/>
         <v>45336</v>
       </c>
-      <c r="AG5" s="126">
+      <c r="AG5" s="120">
         <f t="shared" si="0"/>
         <v>45337</v>
       </c>
-      <c r="AH5" s="126">
+      <c r="AH5" s="120">
         <f t="shared" si="0"/>
         <v>45338</v>
       </c>
-      <c r="AI5" s="126">
+      <c r="AI5" s="120">
         <f t="shared" si="0"/>
         <v>45339</v>
       </c>
-      <c r="AJ5" s="127">
+      <c r="AJ5" s="121">
         <f t="shared" si="0"/>
         <v>45340</v>
       </c>
-      <c r="AK5" s="125">
+      <c r="AK5" s="119">
         <f>AJ5+1</f>
         <v>45341</v>
       </c>
-      <c r="AL5" s="126">
+      <c r="AL5" s="120">
         <f>AK5+1</f>
         <v>45342</v>
       </c>
-      <c r="AM5" s="126">
+      <c r="AM5" s="120">
         <f t="shared" si="0"/>
         <v>45343</v>
       </c>
-      <c r="AN5" s="126">
+      <c r="AN5" s="120">
         <f t="shared" si="0"/>
         <v>45344</v>
       </c>
-      <c r="AO5" s="126">
+      <c r="AO5" s="120">
         <f t="shared" si="0"/>
         <v>45345</v>
       </c>
-      <c r="AP5" s="126">
+      <c r="AP5" s="120">
         <f t="shared" si="0"/>
         <v>45346</v>
       </c>
-      <c r="AQ5" s="127">
+      <c r="AQ5" s="121">
         <f t="shared" si="0"/>
         <v>45347</v>
       </c>
-      <c r="AR5" s="125">
+      <c r="AR5" s="119">
         <f>AQ5+1</f>
         <v>45348</v>
       </c>
-      <c r="AS5" s="126">
+      <c r="AS5" s="120">
         <f>AR5+1</f>
         <v>45349</v>
       </c>
-      <c r="AT5" s="126">
+      <c r="AT5" s="120">
         <f t="shared" si="0"/>
         <v>45350</v>
       </c>
-      <c r="AU5" s="126">
+      <c r="AU5" s="120">
         <f t="shared" si="0"/>
         <v>45351</v>
       </c>
-      <c r="AV5" s="126">
+      <c r="AV5" s="120">
         <f t="shared" si="0"/>
         <v>45352</v>
       </c>
-      <c r="AW5" s="126">
+      <c r="AW5" s="120">
         <f t="shared" si="0"/>
         <v>45353</v>
       </c>
-      <c r="AX5" s="127">
+      <c r="AX5" s="121">
         <f t="shared" si="0"/>
         <v>45354</v>
       </c>
-      <c r="AY5" s="125">
+      <c r="AY5" s="119">
         <f>AX5+1</f>
         <v>45355</v>
       </c>
-      <c r="AZ5" s="126">
+      <c r="AZ5" s="120">
         <f>AY5+1</f>
         <v>45356</v>
       </c>
-      <c r="BA5" s="126">
+      <c r="BA5" s="120">
         <f t="shared" ref="BA5:BE5" si="1">AZ5+1</f>
         <v>45357</v>
       </c>
-      <c r="BB5" s="126">
+      <c r="BB5" s="120">
         <f t="shared" si="1"/>
         <v>45358</v>
       </c>
-      <c r="BC5" s="126">
+      <c r="BC5" s="120">
         <f t="shared" si="1"/>
         <v>45359</v>
       </c>
-      <c r="BD5" s="126">
+      <c r="BD5" s="120">
         <f t="shared" si="1"/>
         <v>45360</v>
       </c>
-      <c r="BE5" s="127">
+      <c r="BE5" s="121">
         <f t="shared" si="1"/>
         <v>45361</v>
       </c>
-      <c r="BF5" s="125">
+      <c r="BF5" s="119">
         <f>BE5+1</f>
         <v>45362</v>
       </c>
-      <c r="BG5" s="126">
+      <c r="BG5" s="120">
         <f>BF5+1</f>
         <v>45363</v>
       </c>
-      <c r="BH5" s="126">
+      <c r="BH5" s="120">
         <f t="shared" ref="BH5:BL5" si="2">BG5+1</f>
         <v>45364</v>
       </c>
-      <c r="BI5" s="126">
+      <c r="BI5" s="120">
         <f t="shared" si="2"/>
         <v>45365</v>
       </c>
-      <c r="BJ5" s="126">
+      <c r="BJ5" s="120">
         <f t="shared" si="2"/>
         <v>45366</v>
       </c>
-      <c r="BK5" s="126">
+      <c r="BK5" s="120">
         <f t="shared" si="2"/>
         <v>45367</v>
       </c>
-      <c r="BL5" s="127">
+      <c r="BL5" s="121">
         <f t="shared" si="2"/>
         <v>45368</v>
       </c>
-      <c r="BM5" s="125">
+      <c r="BM5" s="119">
         <f>BL5+1</f>
         <v>45369</v>
       </c>
-      <c r="BN5" s="126">
+      <c r="BN5" s="120">
         <f>BM5+1</f>
         <v>45370</v>
       </c>
-      <c r="BO5" s="126">
+      <c r="BO5" s="120">
         <f t="shared" ref="BO5:DZ5" si="3">BN5+1</f>
         <v>45371</v>
       </c>
-      <c r="BP5" s="126">
+      <c r="BP5" s="120">
         <f t="shared" si="3"/>
         <v>45372</v>
       </c>
-      <c r="BQ5" s="126">
+      <c r="BQ5" s="120">
         <f t="shared" si="3"/>
         <v>45373</v>
       </c>
-      <c r="BR5" s="126">
+      <c r="BR5" s="120">
         <f t="shared" si="3"/>
         <v>45374</v>
       </c>
-      <c r="BS5" s="127">
+      <c r="BS5" s="121">
         <f t="shared" si="3"/>
         <v>45375</v>
       </c>
-      <c r="BT5" s="125">
+      <c r="BT5" s="119">
         <f t="shared" si="3"/>
         <v>45376</v>
       </c>
-      <c r="BU5" s="126">
+      <c r="BU5" s="120">
         <f t="shared" si="3"/>
         <v>45377</v>
       </c>
-      <c r="BV5" s="126">
+      <c r="BV5" s="120">
         <f t="shared" si="3"/>
         <v>45378</v>
       </c>
-      <c r="BW5" s="126">
+      <c r="BW5" s="120">
         <f t="shared" si="3"/>
         <v>45379</v>
       </c>
-      <c r="BX5" s="126">
+      <c r="BX5" s="120">
         <f t="shared" si="3"/>
         <v>45380</v>
       </c>
-      <c r="BY5" s="126">
+      <c r="BY5" s="120">
         <f t="shared" si="3"/>
         <v>45381</v>
       </c>
-      <c r="BZ5" s="127">
+      <c r="BZ5" s="121">
         <f t="shared" si="3"/>
         <v>45382</v>
       </c>
-      <c r="CA5" s="125">
+      <c r="CA5" s="119">
         <f t="shared" si="3"/>
         <v>45383</v>
       </c>
-      <c r="CB5" s="126">
+      <c r="CB5" s="120">
         <f t="shared" si="3"/>
         <v>45384</v>
       </c>
-      <c r="CC5" s="126">
+      <c r="CC5" s="120">
         <f t="shared" si="3"/>
         <v>45385</v>
       </c>
-      <c r="CD5" s="126">
+      <c r="CD5" s="120">
         <f t="shared" si="3"/>
         <v>45386</v>
       </c>
-      <c r="CE5" s="126">
+      <c r="CE5" s="120">
         <f t="shared" si="3"/>
         <v>45387</v>
       </c>
-      <c r="CF5" s="126">
+      <c r="CF5" s="120">
         <f t="shared" si="3"/>
         <v>45388</v>
       </c>
-      <c r="CG5" s="127">
+      <c r="CG5" s="121">
         <f t="shared" si="3"/>
         <v>45389</v>
       </c>
-      <c r="CH5" s="125">
+      <c r="CH5" s="119">
         <f t="shared" si="3"/>
         <v>45390</v>
       </c>
-      <c r="CI5" s="126">
+      <c r="CI5" s="120">
         <f t="shared" si="3"/>
         <v>45391</v>
       </c>
-      <c r="CJ5" s="126">
+      <c r="CJ5" s="120">
         <f t="shared" si="3"/>
         <v>45392</v>
       </c>
-      <c r="CK5" s="126">
+      <c r="CK5" s="120">
         <f t="shared" si="3"/>
         <v>45393</v>
       </c>
-      <c r="CL5" s="126">
+      <c r="CL5" s="120">
         <f t="shared" si="3"/>
         <v>45394</v>
       </c>
-      <c r="CM5" s="126">
+      <c r="CM5" s="120">
         <f t="shared" si="3"/>
         <v>45395</v>
       </c>
-      <c r="CN5" s="127">
+      <c r="CN5" s="121">
         <f t="shared" si="3"/>
         <v>45396</v>
       </c>
-      <c r="CO5" s="125">
+      <c r="CO5" s="119">
         <f t="shared" si="3"/>
         <v>45397</v>
       </c>
-      <c r="CP5" s="126">
+      <c r="CP5" s="120">
         <f t="shared" si="3"/>
         <v>45398</v>
       </c>
-      <c r="CQ5" s="126">
+      <c r="CQ5" s="120">
         <f t="shared" si="3"/>
         <v>45399</v>
       </c>
-      <c r="CR5" s="126">
+      <c r="CR5" s="120">
         <f t="shared" si="3"/>
         <v>45400</v>
       </c>
-      <c r="CS5" s="126">
+      <c r="CS5" s="120">
         <f t="shared" si="3"/>
         <v>45401</v>
       </c>
-      <c r="CT5" s="126">
+      <c r="CT5" s="120">
         <f t="shared" si="3"/>
         <v>45402</v>
       </c>
-      <c r="CU5" s="127">
+      <c r="CU5" s="121">
         <f t="shared" si="3"/>
         <v>45403</v>
       </c>
-      <c r="CV5" s="125">
+      <c r="CV5" s="119">
         <f t="shared" si="3"/>
         <v>45404</v>
       </c>
-      <c r="CW5" s="126">
+      <c r="CW5" s="120">
         <f t="shared" si="3"/>
         <v>45405</v>
       </c>
-      <c r="CX5" s="126">
+      <c r="CX5" s="120">
         <f t="shared" si="3"/>
         <v>45406</v>
       </c>
-      <c r="CY5" s="126">
+      <c r="CY5" s="120">
         <f t="shared" si="3"/>
         <v>45407</v>
       </c>
-      <c r="CZ5" s="126">
+      <c r="CZ5" s="120">
         <f t="shared" si="3"/>
         <v>45408</v>
       </c>
-      <c r="DA5" s="126">
+      <c r="DA5" s="120">
         <f t="shared" si="3"/>
         <v>45409</v>
       </c>
-      <c r="DB5" s="127">
+      <c r="DB5" s="121">
         <f t="shared" si="3"/>
         <v>45410</v>
       </c>
-      <c r="DC5" s="125">
+      <c r="DC5" s="119">
         <f t="shared" si="3"/>
         <v>45411</v>
       </c>
-      <c r="DD5" s="126">
+      <c r="DD5" s="120">
         <f t="shared" si="3"/>
         <v>45412</v>
       </c>
-      <c r="DE5" s="126">
+      <c r="DE5" s="120">
         <f t="shared" si="3"/>
         <v>45413</v>
       </c>
-      <c r="DF5" s="126">
+      <c r="DF5" s="120">
         <f t="shared" si="3"/>
         <v>45414</v>
       </c>
-      <c r="DG5" s="126">
+      <c r="DG5" s="120">
         <f t="shared" si="3"/>
         <v>45415</v>
       </c>
-      <c r="DH5" s="126">
+      <c r="DH5" s="120">
         <f t="shared" si="3"/>
         <v>45416</v>
       </c>
-      <c r="DI5" s="127">
+      <c r="DI5" s="121">
         <f t="shared" si="3"/>
         <v>45417</v>
       </c>
-      <c r="DJ5" s="125">
+      <c r="DJ5" s="119">
         <f t="shared" si="3"/>
         <v>45418</v>
       </c>
-      <c r="DK5" s="126">
+      <c r="DK5" s="120">
         <f t="shared" si="3"/>
         <v>45419</v>
       </c>
-      <c r="DL5" s="126">
+      <c r="DL5" s="120">
         <f t="shared" si="3"/>
         <v>45420</v>
       </c>
-      <c r="DM5" s="126">
+      <c r="DM5" s="120">
         <f t="shared" si="3"/>
         <v>45421</v>
       </c>
-      <c r="DN5" s="126">
+      <c r="DN5" s="120">
         <f t="shared" si="3"/>
         <v>45422</v>
       </c>
-      <c r="DO5" s="126">
+      <c r="DO5" s="120">
         <f t="shared" si="3"/>
         <v>45423</v>
       </c>
-      <c r="DP5" s="127">
+      <c r="DP5" s="121">
         <f t="shared" si="3"/>
         <v>45424</v>
       </c>
-      <c r="DQ5" s="125">
+      <c r="DQ5" s="119">
         <f t="shared" si="3"/>
         <v>45425</v>
       </c>
-      <c r="DR5" s="126">
+      <c r="DR5" s="120">
         <f t="shared" si="3"/>
         <v>45426</v>
       </c>
-      <c r="DS5" s="126">
+      <c r="DS5" s="120">
         <f t="shared" si="3"/>
         <v>45427</v>
       </c>
-      <c r="DT5" s="126">
+      <c r="DT5" s="120">
         <f t="shared" si="3"/>
         <v>45428</v>
       </c>
-      <c r="DU5" s="126">
+      <c r="DU5" s="120">
         <f t="shared" si="3"/>
         <v>45429</v>
       </c>
-      <c r="DV5" s="126">
+      <c r="DV5" s="120">
         <f t="shared" si="3"/>
         <v>45430</v>
       </c>
-      <c r="DW5" s="127">
+      <c r="DW5" s="121">
         <f t="shared" si="3"/>
         <v>45431</v>
       </c>
-      <c r="DX5" s="125">
+      <c r="DX5" s="119">
         <f t="shared" si="3"/>
         <v>45432</v>
       </c>
-      <c r="DY5" s="126">
+      <c r="DY5" s="120">
         <f t="shared" si="3"/>
         <v>45433</v>
       </c>
-      <c r="DZ5" s="126">
+      <c r="DZ5" s="120">
         <f t="shared" si="3"/>
         <v>45434</v>
       </c>
-      <c r="EA5" s="126">
+      <c r="EA5" s="120">
         <f t="shared" ref="EA5:ED5" si="4">DZ5+1</f>
         <v>45435</v>
       </c>
-      <c r="EB5" s="126">
+      <c r="EB5" s="120">
         <f t="shared" si="4"/>
         <v>45436</v>
       </c>
-      <c r="EC5" s="126">
+      <c r="EC5" s="120">
         <f t="shared" si="4"/>
         <v>45437</v>
       </c>
-      <c r="ED5" s="127">
+      <c r="ED5" s="121">
         <f t="shared" si="4"/>
         <v>45438</v>
       </c>
@@ -20299,16 +20355,16 @@
     <mergeCell ref="CV4:DB4"/>
     <mergeCell ref="DC4:DI4"/>
     <mergeCell ref="BM4:BS4"/>
+    <mergeCell ref="AD4:AJ4"/>
+    <mergeCell ref="AK4:AQ4"/>
+    <mergeCell ref="AR4:AX4"/>
+    <mergeCell ref="AY4:BE4"/>
+    <mergeCell ref="BF4:BL4"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="I4:O4"/>
     <mergeCell ref="P4:V4"/>
     <mergeCell ref="W4:AC4"/>
-    <mergeCell ref="AD4:AJ4"/>
-    <mergeCell ref="AK4:AQ4"/>
-    <mergeCell ref="AR4:AX4"/>
-    <mergeCell ref="AY4:BE4"/>
-    <mergeCell ref="BF4:BL4"/>
   </mergeCells>
   <conditionalFormatting sqref="D7:D13">
     <cfRule type="dataBar" priority="4">

</xml_diff>